<commit_message>
Update PCB files and metadata for new design specifications
</commit_message>
<xml_diff>
--- a/solr-mobile-power-manager/altium/inverter_12V_220V_500W/Fabrication Files/BOM/Bill of Materials-inverter-12v-220v-500w.xlsx
+++ b/solr-mobile-power-manager/altium/inverter_12V_220V_500W/Fabrication Files/BOM/Bill of Materials-inverter-12v-220v-500w.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Stason\Desktop\Projects\pure-sinus\hardware\invertor_12V_220V_500W\Fabrication Files\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Stason\Desktop\Projects\pure-sinus\solr-mobile-power-manager\altium\inverter_12V_220V_500W\Fabrication Files\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D185FF8B-2B11-418E-86F1-086B6D9FA61C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{06FE949A-A35C-4F59-9828-19CA4FCD8D9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12930" yWindow="210" windowWidth="21330" windowHeight="16560" xr2:uid="{74040948-4E8A-4DAE-A94A-E1B2D21422AA}"/>
+    <workbookView xWindow="12930" yWindow="210" windowWidth="21330" windowHeight="16560" xr2:uid="{033733D0-73B0-44EC-AFD0-EA81FA2F3CE5}"/>
   </bookViews>
   <sheets>
     <sheet name="Bill of Materials-inverter-12v-" sheetId="1" r:id="rId1"/>
@@ -134,7 +134,7 @@
     <t>2200uF</t>
   </si>
   <si>
-    <t>C22, C23, C26, C27, C28, C29, C30, C32, C34, C35, C37, C41</t>
+    <t>C22, C23, C26, C27, C28, C29, C30, C32, C34, C35, C37, C41, C43, C44</t>
   </si>
   <si>
     <t>0.1µF</t>
@@ -1047,7 +1047,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8825D65F-5DCC-4535-9FBD-48AB26906792}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{134E2478-E56A-453F-AE16-43CB9BA4C423}">
   <dimension ref="A1:D78"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1213,7 +1213,7 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>31</v>
@@ -2151,6 +2151,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Inverter board improvements: Button connector change and silkscreen fixes
</commit_message>
<xml_diff>
--- a/solr-mobile-power-manager/altium/inverter_12V_220V_500W/Fabrication Files/BOM/Bill of Materials-inverter-12v-220v-500w.xlsx
+++ b/solr-mobile-power-manager/altium/inverter_12V_220V_500W/Fabrication Files/BOM/Bill of Materials-inverter-12v-220v-500w.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Stason\Desktop\Projects\pure-sinus\solr-mobile-power-manager\altium\inverter_12V_220V_500W\Fabrication Files\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{06FE949A-A35C-4F59-9828-19CA4FCD8D9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{708745E9-DB5E-4C37-B8D0-24C3C4663D16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12930" yWindow="210" windowWidth="21330" windowHeight="16560" xr2:uid="{033733D0-73B0-44EC-AFD0-EA81FA2F3CE5}"/>
+    <workbookView xWindow="12930" yWindow="210" windowWidth="21330" windowHeight="16560" xr2:uid="{F2C50F66-27E0-4E9B-8E3F-564F1CB9F602}"/>
   </bookViews>
   <sheets>
     <sheet name="Bill of Materials-inverter-12v-" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="200">
   <si>
     <t>Quantity</t>
   </si>
@@ -317,19 +317,10 @@
     <t>J9</t>
   </si>
   <si>
-    <t>Invertor On/Off</t>
-  </si>
-  <si>
-    <t>J10</t>
-  </si>
-  <si>
-    <t>DC Load On/Off</t>
-  </si>
-  <si>
-    <t>J11</t>
-  </si>
-  <si>
-    <t>LCD On/Off</t>
+    <t>Buttons</t>
+  </si>
+  <si>
+    <t>JST_B4B-XH-AM_(LF)(SN)</t>
   </si>
   <si>
     <t>J12</t>
@@ -341,10 +332,7 @@
     <t>J13</t>
   </si>
   <si>
-    <t>LCD</t>
-  </si>
-  <si>
-    <t>JST_B4B-XH-AM_(LF)(SN)</t>
+    <t>I2C</t>
   </si>
   <si>
     <t>L1</t>
@@ -1047,8 +1035,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{134E2478-E56A-453F-AE16-43CB9BA4C423}">
-  <dimension ref="A1:D78"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58D03913-0BC4-4D50-93D9-036C685BE8C7}">
+  <dimension ref="A1:D76"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.28515625" customWidth="1"/>
@@ -1544,7 +1532,7 @@
         <v>92</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
@@ -1552,10 +1540,10 @@
         <v>1</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>88</v>
@@ -1566,13 +1554,13 @@
         <v>1</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
@@ -1580,13 +1568,13 @@
         <v>1</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>88</v>
+        <v>100</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
@@ -1594,13 +1582,13 @@
         <v>1</v>
       </c>
       <c r="B39" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="C39" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="C39" s="2" t="s">
-        <v>100</v>
-      </c>
       <c r="D39" s="2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
@@ -1608,13 +1596,13 @@
         <v>1</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
@@ -1622,13 +1610,13 @@
         <v>1</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
@@ -1636,13 +1624,13 @@
         <v>1</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
@@ -1650,83 +1638,83 @@
         <v>1</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
@@ -1734,27 +1722,27 @@
         <v>1</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
@@ -1762,60 +1750,60 @@
         <v>1</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>143</v>
+        <v>131</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B55" s="2" t="s">
         <v>144</v>
@@ -1824,12 +1812,12 @@
         <v>145</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B56" s="2" t="s">
         <v>146</v>
@@ -1838,91 +1826,91 @@
         <v>147</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>135</v>
+        <v>148</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B57" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="C57" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="D57" s="2" t="s">
         <v>148</v>
-      </c>
-      <c r="C57" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="D57" s="2" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" s="1">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="B59" s="2" t="s">
         <v>153</v>
       </c>
       <c r="C59" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="D59" s="2" t="s">
         <v>154</v>
-      </c>
-      <c r="D59" s="2" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B60" s="2" t="s">
         <v>155</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>156</v>
+        <v>141</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="1">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="B61" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="C61" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="C61" s="2" t="s">
-        <v>145</v>
-      </c>
       <c r="D61" s="2" t="s">
-        <v>158</v>
+        <v>148</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B62" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="C62" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="C62" s="2" t="s">
-        <v>145</v>
-      </c>
       <c r="D62" s="2" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
@@ -1936,12 +1924,12 @@
         <v>161</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B64" s="2" t="s">
         <v>162</v>
@@ -1950,7 +1938,7 @@
         <v>163</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>152</v>
+        <v>164</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
@@ -1958,27 +1946,27 @@
         <v>1</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
@@ -1986,13 +1974,13 @@
         <v>1</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
@@ -2000,27 +1988,27 @@
         <v>1</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
@@ -2028,27 +2016,27 @@
         <v>1</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
@@ -2056,13 +2044,13 @@
         <v>1</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
@@ -2070,13 +2058,13 @@
         <v>1</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
@@ -2084,13 +2072,13 @@
         <v>1</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
@@ -2098,13 +2086,13 @@
         <v>1</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
@@ -2112,41 +2100,13 @@
         <v>1</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A77" s="1">
-        <v>1</v>
-      </c>
-      <c r="B77" s="2" t="s">
-        <v>198</v>
-      </c>
-      <c r="C77" s="2" t="s">
         <v>199</v>
-      </c>
-      <c r="D77" s="2" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A78" s="1">
-        <v>1</v>
-      </c>
-      <c r="B78" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="C78" s="2" t="s">
-        <v>202</v>
-      </c>
-      <c r="D78" s="2" t="s">
-        <v>203</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Solr button module: implementation
</commit_message>
<xml_diff>
--- a/solr-mobile-power-manager/altium/inverter_12V_220V_500W/Fabrication Files/BOM/Bill of Materials-inverter-12v-220v-500w.xlsx
+++ b/solr-mobile-power-manager/altium/inverter_12V_220V_500W/Fabrication Files/BOM/Bill of Materials-inverter-12v-220v-500w.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Stason\Desktop\Projects\pure-sinus\solr-mobile-power-manager\altium\inverter_12V_220V_500W\Fabrication Files\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{708745E9-DB5E-4C37-B8D0-24C3C4663D16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7B7FDDD4-208F-48FD-BC22-F8C81D577489}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12930" yWindow="210" windowWidth="21330" windowHeight="16560" xr2:uid="{F2C50F66-27E0-4E9B-8E3F-564F1CB9F602}"/>
+    <workbookView xWindow="12930" yWindow="210" windowWidth="21330" windowHeight="16560" xr2:uid="{515DE6AA-EF85-4959-9CF8-47F2BE3693F7}"/>
   </bookViews>
   <sheets>
     <sheet name="Bill of Materials-inverter-12v-" sheetId="1" r:id="rId1"/>
@@ -34,12 +34,15 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="2"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="202">
   <si>
     <t>Quantity</t>
   </si>
@@ -321,6 +324,12 @@
   </si>
   <si>
     <t>JST_B4B-XH-AM_(LF)(SN)</t>
+  </si>
+  <si>
+    <t>J10</t>
+  </si>
+  <si>
+    <t>VH396-02S-010</t>
   </si>
   <si>
     <t>J12</t>
@@ -1035,8 +1044,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58D03913-0BC4-4D50-93D9-036C685BE8C7}">
-  <dimension ref="A1:D76"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B9FBB69-428F-4BC8-AC18-2C271F0BF343}">
+  <dimension ref="A1:D77"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.28515625" customWidth="1"/>
@@ -1546,7 +1555,7 @@
         <v>95</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>88</v>
+        <v>73</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
@@ -1560,7 +1569,7 @@
         <v>97</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
@@ -1574,7 +1583,7 @@
         <v>99</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
@@ -1582,10 +1591,10 @@
         <v>1</v>
       </c>
       <c r="B39" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="C39" s="2" t="s">
         <v>101</v>
-      </c>
-      <c r="C39" s="2" t="s">
-        <v>99</v>
       </c>
       <c r="D39" s="2" t="s">
         <v>102</v>
@@ -1599,10 +1608,10 @@
         <v>103</v>
       </c>
       <c r="C40" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="D40" s="2" t="s">
         <v>104</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
@@ -1610,13 +1619,13 @@
         <v>1</v>
       </c>
       <c r="B41" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C41" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="C41" s="2" t="s">
+      <c r="D41" s="2" t="s">
         <v>107</v>
-      </c>
-      <c r="D41" s="2" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
@@ -1624,10 +1633,10 @@
         <v>1</v>
       </c>
       <c r="B42" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="C42" s="2" t="s">
         <v>109</v>
-      </c>
-      <c r="C42" s="2" t="s">
-        <v>110</v>
       </c>
       <c r="D42" s="2" t="s">
         <v>110</v>
@@ -1644,21 +1653,21 @@
         <v>112</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B44" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="C44" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="C44" s="2" t="s">
+      <c r="D44" s="2" t="s">
         <v>115</v>
-      </c>
-      <c r="D44" s="2" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
@@ -1666,41 +1675,41 @@
         <v>4</v>
       </c>
       <c r="B45" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="C45" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="C45" s="2" t="s">
+      <c r="D45" s="2" t="s">
         <v>118</v>
-      </c>
-      <c r="D45" s="2" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B46" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="C46" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="C46" s="2" t="s">
+      <c r="D46" s="2" t="s">
         <v>121</v>
-      </c>
-      <c r="D46" s="2" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B47" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="C47" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="C47" s="2" t="s">
+      <c r="D47" s="2" t="s">
         <v>124</v>
-      </c>
-      <c r="D47" s="2" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
@@ -1708,13 +1717,13 @@
         <v>1</v>
       </c>
       <c r="B48" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="C48" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="C48" s="2" t="s">
+      <c r="D48" s="2" t="s">
         <v>127</v>
-      </c>
-      <c r="D48" s="2" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
@@ -1722,41 +1731,41 @@
         <v>1</v>
       </c>
       <c r="B49" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="C49" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="C49" s="2" t="s">
+      <c r="D49" s="2" t="s">
         <v>130</v>
-      </c>
-      <c r="D49" s="2" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B50" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="C50" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="C50" s="2" t="s">
+      <c r="D50" s="2" t="s">
         <v>133</v>
-      </c>
-      <c r="D50" s="2" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B51" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="C51" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="C51" s="2" t="s">
+      <c r="D51" s="2" t="s">
         <v>136</v>
-      </c>
-      <c r="D51" s="2" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
@@ -1770,26 +1779,26 @@
         <v>138</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B53" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="C53" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="C53" s="2" t="s">
+      <c r="D53" s="2" t="s">
         <v>141</v>
-      </c>
-      <c r="D53" s="2" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B54" s="2" t="s">
         <v>142</v>
@@ -1798,7 +1807,7 @@
         <v>143</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
@@ -1812,12 +1821,12 @@
         <v>145</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B56" s="2" t="s">
         <v>146</v>
@@ -1826,7 +1835,7 @@
         <v>147</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>148</v>
+        <v>133</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
@@ -1834,18 +1843,18 @@
         <v>3</v>
       </c>
       <c r="B57" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="C57" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="C57" s="2" t="s">
+      <c r="D57" s="2" t="s">
         <v>150</v>
-      </c>
-      <c r="D57" s="2" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B58" s="2" t="s">
         <v>151</v>
@@ -1854,49 +1863,49 @@
         <v>152</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" s="1">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B59" s="2" t="s">
         <v>153</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>141</v>
+        <v>154</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" s="1">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="B60" s="2" t="s">
         <v>155</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>157</v>
+        <v>143</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
@@ -1910,7 +1919,7 @@
         <v>159</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
@@ -1924,12 +1933,12 @@
         <v>161</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B64" s="2" t="s">
         <v>162</v>
@@ -1938,18 +1947,18 @@
         <v>163</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B65" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C65" s="2" t="s">
         <v>165</v>
-      </c>
-      <c r="C65" s="2" t="s">
-        <v>166</v>
       </c>
       <c r="D65" s="2" t="s">
         <v>166</v>
@@ -1966,7 +1975,7 @@
         <v>168</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
@@ -1974,13 +1983,13 @@
         <v>1</v>
       </c>
       <c r="B67" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="C67" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="C67" s="2" t="s">
+      <c r="D67" s="2" t="s">
         <v>171</v>
-      </c>
-      <c r="D67" s="2" t="s">
-        <v>172</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
@@ -1988,41 +1997,41 @@
         <v>1</v>
       </c>
       <c r="B68" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="C68" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="C68" s="2" t="s">
+      <c r="D68" s="2" t="s">
         <v>174</v>
-      </c>
-      <c r="D68" s="2" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B69" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C69" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="C69" s="2" t="s">
+      <c r="D69" s="2" t="s">
         <v>177</v>
-      </c>
-      <c r="D69" s="2" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B70" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="C70" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="C70" s="2" t="s">
+      <c r="D70" s="2" t="s">
         <v>180</v>
-      </c>
-      <c r="D70" s="2" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
@@ -2030,13 +2039,13 @@
         <v>1</v>
       </c>
       <c r="B71" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C71" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="C71" s="2" t="s">
+      <c r="D71" s="2" t="s">
         <v>183</v>
-      </c>
-      <c r="D71" s="2" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
@@ -2044,13 +2053,13 @@
         <v>1</v>
       </c>
       <c r="B72" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="C72" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="C72" s="2" t="s">
+      <c r="D72" s="2" t="s">
         <v>186</v>
-      </c>
-      <c r="D72" s="2" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
@@ -2058,13 +2067,13 @@
         <v>1</v>
       </c>
       <c r="B73" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="C73" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="C73" s="2" t="s">
+      <c r="D73" s="2" t="s">
         <v>189</v>
-      </c>
-      <c r="D73" s="2" t="s">
-        <v>190</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
@@ -2072,13 +2081,13 @@
         <v>1</v>
       </c>
       <c r="B74" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="C74" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="C74" s="2" t="s">
+      <c r="D74" s="2" t="s">
         <v>192</v>
-      </c>
-      <c r="D74" s="2" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
@@ -2086,13 +2095,13 @@
         <v>1</v>
       </c>
       <c r="B75" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C75" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="C75" s="2" t="s">
+      <c r="D75" s="2" t="s">
         <v>195</v>
-      </c>
-      <c r="D75" s="2" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
@@ -2100,13 +2109,27 @@
         <v>1</v>
       </c>
       <c r="B76" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="C76" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="C76" s="2" t="s">
+      <c r="D76" s="2" t="s">
         <v>198</v>
       </c>
-      <c r="D76" s="2" t="s">
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A77" s="1">
+        <v>1</v>
+      </c>
+      <c r="B77" s="2" t="s">
         <v>199</v>
+      </c>
+      <c r="C77" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="D77" s="2" t="s">
+        <v>201</v>
       </c>
     </row>
   </sheetData>

</xml_diff>